<commit_message>
Mise à jour du mapping suite évolution ML 7260e39f5636ea5bf89ffb7737d283c660afe1b4
</commit_message>
<xml_diff>
--- a/MAJImagingLM/ig/FRSectionSupportingInformationLMCDAFHIR.xlsx
+++ b/MAJImagingLM/ig/FRSectionSupportingInformationLMCDAFHIR.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="71">
   <si>
     <t>Property</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-10T13:41:51+00:00</t>
+    <t>2026-09-14T09:02:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -149,6 +149,9 @@
     <t>FRLMSupportingInformation.entry.historyOfPastIllness</t>
   </si>
   <si>
+    <t>FRLMObservation</t>
+  </si>
+  <si>
     <t>Section.entry.observation</t>
   </si>
   <si>
@@ -194,13 +197,16 @@
     <t>Observation</t>
   </si>
   <si>
+    <t>FRLMCondition</t>
+  </si>
+  <si>
+    <t>FRConditionDocument</t>
+  </si>
+  <si>
     <t>FRObservationContraIndicationsDocument</t>
   </si>
   <si>
     <t>FRLMSupportingInformation.entry.condition</t>
-  </si>
-  <si>
-    <t>FRConditionDocument</t>
   </si>
   <si>
     <t>FRObservationPregnancyDocument</t>
@@ -572,60 +578,62 @@
       <c r="A7" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" t="s" s="2">
+        <v>44</v>
+      </c>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -635,7 +643,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -666,7 +674,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -681,10 +689,10 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -696,7 +704,7 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -709,7 +717,7 @@
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -722,65 +730,69 @@
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="B8" s="2"/>
+      <c r="B8" t="s" s="2">
+        <v>44</v>
+      </c>
       <c r="C8" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="B9" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="B9" t="s" s="2">
+        <v>60</v>
+      </c>
       <c r="C9" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s" s="2">
         <v>59</v>
@@ -788,32 +800,47 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="2">
+        <v>48</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s" s="2">
+        <v>58</v>
+      </c>
+      <c r="E13" t="s" s="2">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -854,7 +881,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -869,22 +896,22 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -897,85 +924,85 @@
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E11" s="2"/>
     </row>

</xml_diff>